<commit_message>
Added code for marketplace
</commit_message>
<xml_diff>
--- a/data/DrugPageData.xlsx
+++ b/data/DrugPageData.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="19" documentId="11_E0A3203620397D6A206102BBF0179E13A12C073D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25851A19-3030-484F-BD75-E93848823E1B}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plans" sheetId="1" r:id="rId1"/>
@@ -238,10 +238,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -567,16 +563,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F23"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.796875" customWidth="1"/>
-    <col min="2" max="3" width="6.796875" customWidth="1"/>
-    <col min="4" max="4" width="40.796875" customWidth="1"/>
+    <col min="1" max="1" width="5.75" customWidth="1"/>
+    <col min="2" max="3" width="6.75" customWidth="1"/>
+    <col min="4" max="4" width="40.75" customWidth="1"/>
     <col min="5" max="5" width="70.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="120.796875" customWidth="1"/>
+    <col min="6" max="6" width="120.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -596,7 +592,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -616,7 +612,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -636,7 +632,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -656,7 +652,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -676,7 +672,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -696,7 +692,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -716,7 +712,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -736,7 +732,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -756,7 +752,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -776,7 +772,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -796,7 +792,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -816,7 +812,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -836,7 +832,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -856,7 +852,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -876,7 +872,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -896,7 +892,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -916,7 +912,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>14</v>
       </c>
@@ -936,7 +932,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>14</v>
       </c>
@@ -956,7 +952,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -976,7 +972,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>14</v>
       </c>
@@ -996,7 +992,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>14</v>
       </c>
@@ -1016,7 +1012,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>14</v>
       </c>

</xml_diff>